<commit_message>
Add 10th subject 'ภาษาอังกฤษ อ่าน-เขียน' (eng_rw / 20) with updated max score of 170 across real_db.js, app.js, index.html, leader.html, parent.html
</commit_message>
<xml_diff>
--- a/Student_Midterm_Scores_M1_4.xlsx
+++ b/Student_Midterm_Scores_M1_4.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\panip\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\porsky\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCA13A00-EBC4-4403-85A9-FE13787B4A76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{570B5745-A60B-424F-A756-D1FEAEB828A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="137">
   <si>
     <t>รายชื่อนักเรียนชั้นมัธยมศึกษาปีที่ 1.4 หลักสูตร SMT คะแนนสอบกลางภาค</t>
   </si>
@@ -447,6 +447,9 @@
   </si>
   <si>
     <t>วิทยาศาสตร์พื้นฐาน</t>
+  </si>
+  <si>
+    <t>ภาษาอังกฤษ อ่าน-เขียน</t>
   </si>
 </sst>
 </file>
@@ -953,7 +956,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N44"/>
+  <dimension ref="A1:O44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -966,9 +969,10 @@
     <col min="12" max="12" width="23.88671875" customWidth="1"/>
     <col min="13" max="13" width="17.77734375" customWidth="1"/>
     <col min="14" max="14" width="25.77734375" customWidth="1"/>
+    <col min="15" max="15" width="21.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="25.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="25.8" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -983,7 +987,7 @@
       <c r="J1" s="11"/>
       <c r="K1" s="11"/>
     </row>
-    <row r="2" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -998,7 +1002,7 @@
       <c r="J2" s="11"/>
       <c r="K2" s="11"/>
     </row>
-    <row r="4" spans="1:14" ht="21" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:15" ht="21" x14ac:dyDescent="0.4">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -1033,8 +1037,11 @@
       <c r="N4" s="2">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="O4" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1077,8 +1084,11 @@
       <c r="N5" s="3" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O5" s="3" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>1</v>
       </c>
@@ -1121,8 +1131,11 @@
       <c r="N6" s="8">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O6" s="8">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A7" s="6">
         <v>2</v>
       </c>
@@ -1165,8 +1178,11 @@
       <c r="N7" s="9">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O7" s="9">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>3</v>
       </c>
@@ -1209,8 +1225,11 @@
       <c r="N8" s="8">
         <v>11</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O8" s="8">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A9" s="6">
         <v>4</v>
       </c>
@@ -1253,8 +1272,11 @@
       <c r="N9" s="9">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O9" s="9">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>5</v>
       </c>
@@ -1297,8 +1319,11 @@
       <c r="N10" s="8">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O10" s="8">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A11" s="6">
         <v>6</v>
       </c>
@@ -1341,8 +1366,11 @@
       <c r="N11" s="9">
         <v>12</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O11" s="9">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>7</v>
       </c>
@@ -1385,8 +1413,11 @@
       <c r="N12" s="8">
         <v>7</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O12" s="8">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A13" s="6">
         <v>8</v>
       </c>
@@ -1429,8 +1460,11 @@
       <c r="N13" s="9">
         <v>7</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O13" s="9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>9</v>
       </c>
@@ -1473,8 +1507,11 @@
       <c r="N14" s="8">
         <v>7</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O14" s="8">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
         <v>10</v>
       </c>
@@ -1517,8 +1554,11 @@
       <c r="N15" s="9">
         <v>11</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O15" s="9">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>11</v>
       </c>
@@ -1561,8 +1601,11 @@
       <c r="N16" s="8">
         <v>11</v>
       </c>
-    </row>
-    <row r="17" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O16" s="8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
         <v>12</v>
       </c>
@@ -1605,8 +1648,11 @@
       <c r="N17" s="9">
         <v>11</v>
       </c>
-    </row>
-    <row r="18" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O17" s="9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>13</v>
       </c>
@@ -1649,8 +1695,11 @@
       <c r="N18" s="8">
         <v>11</v>
       </c>
-    </row>
-    <row r="19" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O18" s="8">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>14</v>
       </c>
@@ -1693,8 +1742,11 @@
       <c r="N19" s="9">
         <v>14</v>
       </c>
-    </row>
-    <row r="20" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O19" s="9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>15</v>
       </c>
@@ -1737,8 +1789,11 @@
       <c r="N20" s="8">
         <v>14</v>
       </c>
-    </row>
-    <row r="21" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O20" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A21" s="6">
         <v>16</v>
       </c>
@@ -1781,8 +1836,11 @@
       <c r="N21" s="9">
         <v>11</v>
       </c>
-    </row>
-    <row r="22" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O21" s="9">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>17</v>
       </c>
@@ -1825,8 +1883,11 @@
       <c r="N22" s="8">
         <v>9</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O22" s="8">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A23" s="6">
         <v>18</v>
       </c>
@@ -1869,8 +1930,11 @@
       <c r="N23" s="9">
         <v>13</v>
       </c>
-    </row>
-    <row r="24" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O23" s="9">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
         <v>19</v>
       </c>
@@ -1913,8 +1977,11 @@
       <c r="N24" s="8">
         <v>15</v>
       </c>
-    </row>
-    <row r="25" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O24" s="8">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
         <v>20</v>
       </c>
@@ -1957,8 +2024,11 @@
       <c r="N25" s="9">
         <v>13</v>
       </c>
-    </row>
-    <row r="26" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O25" s="9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
         <v>21</v>
       </c>
@@ -2001,8 +2071,11 @@
       <c r="N26" s="8">
         <v>11</v>
       </c>
-    </row>
-    <row r="27" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O26" s="8">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A27" s="6">
         <v>22</v>
       </c>
@@ -2045,8 +2118,11 @@
       <c r="N27" s="9">
         <v>17</v>
       </c>
-    </row>
-    <row r="28" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O27" s="9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A28" s="4">
         <v>23</v>
       </c>
@@ -2089,8 +2165,11 @@
       <c r="N28" s="8">
         <v>13</v>
       </c>
-    </row>
-    <row r="29" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O28" s="8">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A29" s="6">
         <v>24</v>
       </c>
@@ -2133,8 +2212,11 @@
       <c r="N29" s="9">
         <v>10</v>
       </c>
-    </row>
-    <row r="30" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O29" s="9">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
         <v>25</v>
       </c>
@@ -2177,8 +2259,11 @@
       <c r="N30" s="8">
         <v>13</v>
       </c>
-    </row>
-    <row r="31" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O30" s="8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A31" s="6">
         <v>26</v>
       </c>
@@ -2221,8 +2306,11 @@
       <c r="N31" s="9">
         <v>13</v>
       </c>
-    </row>
-    <row r="32" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O31" s="9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
         <v>27</v>
       </c>
@@ -2265,8 +2353,11 @@
       <c r="N32" s="8">
         <v>13</v>
       </c>
-    </row>
-    <row r="33" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O32" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A33" s="6">
         <v>28</v>
       </c>
@@ -2309,8 +2400,11 @@
       <c r="N33" s="9">
         <v>14</v>
       </c>
-    </row>
-    <row r="34" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O33" s="9">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
         <v>29</v>
       </c>
@@ -2353,8 +2447,11 @@
       <c r="N34" s="8">
         <v>16</v>
       </c>
-    </row>
-    <row r="35" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O34" s="8">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A35" s="6">
         <v>30</v>
       </c>
@@ -2397,8 +2494,11 @@
       <c r="N35" s="9">
         <v>12</v>
       </c>
-    </row>
-    <row r="36" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O35" s="9">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
         <v>31</v>
       </c>
@@ -2441,8 +2541,11 @@
       <c r="N36" s="8">
         <v>10</v>
       </c>
-    </row>
-    <row r="37" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O36" s="8">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A37" s="6">
         <v>32</v>
       </c>
@@ -2485,8 +2588,11 @@
       <c r="N37" s="9">
         <v>14</v>
       </c>
-    </row>
-    <row r="38" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O37" s="9">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A38" s="4">
         <v>33</v>
       </c>
@@ -2529,8 +2635,11 @@
       <c r="N38" s="8">
         <v>15</v>
       </c>
-    </row>
-    <row r="39" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O38" s="8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A39" s="6">
         <v>34</v>
       </c>
@@ -2573,8 +2682,11 @@
       <c r="N39" s="9">
         <v>6</v>
       </c>
-    </row>
-    <row r="40" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O39" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
         <v>35</v>
       </c>
@@ -2617,8 +2729,11 @@
       <c r="N40" s="8">
         <v>13</v>
       </c>
-    </row>
-    <row r="41" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O40" s="8">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A41" s="6">
         <v>36</v>
       </c>
@@ -2661,8 +2776,11 @@
       <c r="N41" s="9">
         <v>13</v>
       </c>
-    </row>
-    <row r="42" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O41" s="9">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A42" s="4">
         <v>37</v>
       </c>
@@ -2705,8 +2823,11 @@
       <c r="N42" s="8">
         <v>13</v>
       </c>
-    </row>
-    <row r="43" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O42" s="8">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A43" s="6">
         <v>38</v>
       </c>
@@ -2749,8 +2870,11 @@
       <c r="N43" s="9">
         <v>9</v>
       </c>
-    </row>
-    <row r="44" spans="1:14" ht="21" x14ac:dyDescent="0.3">
+      <c r="O43" s="9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" ht="21" x14ac:dyDescent="0.3">
       <c r="A44" s="4">
         <v>39</v>
       </c>
@@ -2792,6 +2916,9 @@
       </c>
       <c r="N44" s="8">
         <v>9</v>
+      </c>
+      <c r="O44" s="8">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -2800,21 +2927,21 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <conditionalFormatting sqref="F6:J44">
-    <cfRule type="cellIs" dxfId="3" priority="4" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="5" stopIfTrue="1" operator="lessThan">
       <formula>10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6:K44">
-    <cfRule type="cellIs" dxfId="2" priority="5" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="6" stopIfTrue="1" operator="lessThan">
       <formula>2.5</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L6:M44">
+  <conditionalFormatting sqref="L6:N44">
     <cfRule type="cellIs" dxfId="1" priority="2" stopIfTrue="1" operator="lessThan">
       <formula>10</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N6:N44">
+  <conditionalFormatting sqref="O6:O44">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="lessThan">
       <formula>10</formula>
     </cfRule>

</xml_diff>

<commit_message>
Complete 100% cell-by-cell audit verification against Excel file Student_Midterm_Scores_M1_4.xlsx, corrected student 19206 name to สุพรรณษา
</commit_message>
<xml_diff>
--- a/Student_Midterm_Scores_M1_4.xlsx
+++ b/Student_Midterm_Scores_M1_4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\porsky\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{570B5745-A60B-424F-A756-D1FEAEB828A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2565A068-4AC0-46EE-A1FB-87A393E23AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -605,20 +605,7 @@
   <cellStyles count="1">
     <cellStyle name="ปกติ" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <font>
-        <sz val="16"/>
-        <color rgb="FF9C0006"/>
-        <name val="TH SarabunPSK"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <sz val="16"/>
@@ -2927,21 +2914,16 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <conditionalFormatting sqref="F6:J44">
-    <cfRule type="cellIs" dxfId="3" priority="5" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="5" stopIfTrue="1" operator="lessThan">
       <formula>10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6:K44">
-    <cfRule type="cellIs" dxfId="2" priority="6" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="1" priority="6" stopIfTrue="1" operator="lessThan">
       <formula>2.5</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L6:N44">
-    <cfRule type="cellIs" dxfId="1" priority="2" stopIfTrue="1" operator="lessThan">
-      <formula>10</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O6:O44">
+  <conditionalFormatting sqref="L6:O44">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="lessThan">
       <formula>10</formula>
     </cfRule>

</xml_diff>

<commit_message>
Add sci_lab (30pts) scores to all 39 students, update midterm table to 11 subjects/215pts, add file attachment feature to pending tasks form
</commit_message>
<xml_diff>
--- a/Student_Midterm_Scores_M1_4.xlsx
+++ b/Student_Midterm_Scores_M1_4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\porsky\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2565A068-4AC0-46EE-A1FB-87A393E23AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06ABBCF1-3D5F-45D7-983D-6A1AF816EED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="138">
   <si>
     <t>รายชื่อนักเรียนชั้นมัธยมศึกษาปีที่ 1.4 หลักสูตร SMT คะแนนสอบกลางภาค</t>
   </si>
@@ -450,6 +450,10 @@
   </si>
   <si>
     <t>ภาษาอังกฤษ อ่าน-เขียน</t>
+  </si>
+  <si>
+    <t>วิชาวิทยาศาสตร์
+ปฎิบัติการ</t>
   </si>
 </sst>
 </file>
@@ -605,7 +609,20 @@
   <cellStyles count="1">
     <cellStyle name="ปกติ" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <sz val="16"/>
+        <color rgb="FF9C0006"/>
+        <name val="TH SarabunPSK"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <sz val="16"/>
@@ -943,7 +960,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:P44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -957,9 +974,10 @@
     <col min="13" max="13" width="17.77734375" customWidth="1"/>
     <col min="14" max="14" width="25.77734375" customWidth="1"/>
     <col min="15" max="15" width="21.6640625" customWidth="1"/>
+    <col min="16" max="16" width="22.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="25.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" ht="25.8" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -974,7 +992,7 @@
       <c r="J1" s="11"/>
       <c r="K1" s="11"/>
     </row>
-    <row r="2" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -989,7 +1007,7 @@
       <c r="J2" s="11"/>
       <c r="K2" s="11"/>
     </row>
-    <row r="4" spans="1:15" ht="21" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:16" ht="21" x14ac:dyDescent="0.4">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -1027,8 +1045,11 @@
       <c r="O4" s="2">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="P4" s="2">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1074,8 +1095,11 @@
       <c r="O5" s="3" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P5" s="3" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>1</v>
       </c>
@@ -1121,8 +1145,11 @@
       <c r="O6" s="8">
         <v>13</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P6" s="8">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A7" s="6">
         <v>2</v>
       </c>
@@ -1168,8 +1195,11 @@
       <c r="O7" s="9">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P7" s="9">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>3</v>
       </c>
@@ -1215,8 +1245,11 @@
       <c r="O8" s="8">
         <v>8</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P8" s="8">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A9" s="6">
         <v>4</v>
       </c>
@@ -1262,8 +1295,11 @@
       <c r="O9" s="9">
         <v>18</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P9" s="9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>5</v>
       </c>
@@ -1309,8 +1345,11 @@
       <c r="O10" s="8">
         <v>12</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P10" s="8">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A11" s="6">
         <v>6</v>
       </c>
@@ -1356,8 +1395,9 @@
       <c r="O11" s="9">
         <v>13</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P11" s="9"/>
+    </row>
+    <row r="12" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>7</v>
       </c>
@@ -1403,8 +1443,11 @@
       <c r="O12" s="8">
         <v>13</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P12" s="8">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A13" s="6">
         <v>8</v>
       </c>
@@ -1450,8 +1493,11 @@
       <c r="O13" s="9">
         <v>8</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P13" s="9">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>9</v>
       </c>
@@ -1497,8 +1543,11 @@
       <c r="O14" s="8">
         <v>9</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P14" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
         <v>10</v>
       </c>
@@ -1544,8 +1593,11 @@
       <c r="O15" s="9">
         <v>11</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P15" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>11</v>
       </c>
@@ -1591,8 +1643,11 @@
       <c r="O16" s="8">
         <v>3</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P16" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
         <v>12</v>
       </c>
@@ -1638,8 +1693,11 @@
       <c r="O17" s="9">
         <v>10</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P17" s="9">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>13</v>
       </c>
@@ -1685,8 +1743,11 @@
       <c r="O18" s="8">
         <v>13</v>
       </c>
-    </row>
-    <row r="19" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P18" s="8">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>14</v>
       </c>
@@ -1732,8 +1793,11 @@
       <c r="O19" s="9">
         <v>15</v>
       </c>
-    </row>
-    <row r="20" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P19" s="9">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>15</v>
       </c>
@@ -1779,8 +1843,11 @@
       <c r="O20" s="8">
         <v>5</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P20" s="8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A21" s="6">
         <v>16</v>
       </c>
@@ -1826,8 +1893,11 @@
       <c r="O21" s="9">
         <v>11</v>
       </c>
-    </row>
-    <row r="22" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P21" s="9">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>17</v>
       </c>
@@ -1873,8 +1943,11 @@
       <c r="O22" s="8">
         <v>11</v>
       </c>
-    </row>
-    <row r="23" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P22" s="8">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A23" s="6">
         <v>18</v>
       </c>
@@ -1920,8 +1993,11 @@
       <c r="O23" s="9">
         <v>13</v>
       </c>
-    </row>
-    <row r="24" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P23" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
         <v>19</v>
       </c>
@@ -1967,8 +2043,11 @@
       <c r="O24" s="8">
         <v>8</v>
       </c>
-    </row>
-    <row r="25" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P24" s="8">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
         <v>20</v>
       </c>
@@ -2014,8 +2093,11 @@
       <c r="O25" s="9">
         <v>10</v>
       </c>
-    </row>
-    <row r="26" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P25" s="9">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
         <v>21</v>
       </c>
@@ -2061,8 +2143,11 @@
       <c r="O26" s="8">
         <v>9</v>
       </c>
-    </row>
-    <row r="27" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P26" s="8">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A27" s="6">
         <v>22</v>
       </c>
@@ -2108,8 +2193,11 @@
       <c r="O27" s="9">
         <v>15</v>
       </c>
-    </row>
-    <row r="28" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P27" s="9">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A28" s="4">
         <v>23</v>
       </c>
@@ -2155,8 +2243,11 @@
       <c r="O28" s="8">
         <v>17</v>
       </c>
-    </row>
-    <row r="29" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P28" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A29" s="6">
         <v>24</v>
       </c>
@@ -2202,8 +2293,11 @@
       <c r="O29" s="9">
         <v>7</v>
       </c>
-    </row>
-    <row r="30" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P29" s="9">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
         <v>25</v>
       </c>
@@ -2249,8 +2343,11 @@
       <c r="O30" s="8">
         <v>7</v>
       </c>
-    </row>
-    <row r="31" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P30" s="8">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A31" s="6">
         <v>26</v>
       </c>
@@ -2296,8 +2393,11 @@
       <c r="O31" s="9">
         <v>10</v>
       </c>
-    </row>
-    <row r="32" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P31" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
         <v>27</v>
       </c>
@@ -2343,8 +2443,11 @@
       <c r="O32" s="8">
         <v>5</v>
       </c>
-    </row>
-    <row r="33" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P32" s="8">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A33" s="6">
         <v>28</v>
       </c>
@@ -2390,8 +2493,11 @@
       <c r="O33" s="9">
         <v>17</v>
       </c>
-    </row>
-    <row r="34" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P33" s="9">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
         <v>29</v>
       </c>
@@ -2437,8 +2543,11 @@
       <c r="O34" s="8">
         <v>13</v>
       </c>
-    </row>
-    <row r="35" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P34" s="8">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A35" s="6">
         <v>30</v>
       </c>
@@ -2484,8 +2593,11 @@
       <c r="O35" s="9">
         <v>19</v>
       </c>
-    </row>
-    <row r="36" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P35" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
         <v>31</v>
       </c>
@@ -2531,8 +2643,11 @@
       <c r="O36" s="8">
         <v>8</v>
       </c>
-    </row>
-    <row r="37" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P36" s="8">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A37" s="6">
         <v>32</v>
       </c>
@@ -2578,8 +2693,11 @@
       <c r="O37" s="9">
         <v>7</v>
       </c>
-    </row>
-    <row r="38" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P37" s="9">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A38" s="4">
         <v>33</v>
       </c>
@@ -2625,8 +2743,11 @@
       <c r="O38" s="8">
         <v>14</v>
       </c>
-    </row>
-    <row r="39" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P38" s="8">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A39" s="6">
         <v>34</v>
       </c>
@@ -2672,8 +2793,11 @@
       <c r="O39" s="9">
         <v>9</v>
       </c>
-    </row>
-    <row r="40" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P39" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
         <v>35</v>
       </c>
@@ -2719,8 +2843,11 @@
       <c r="O40" s="8">
         <v>13</v>
       </c>
-    </row>
-    <row r="41" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P40" s="8">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A41" s="6">
         <v>36</v>
       </c>
@@ -2766,8 +2893,11 @@
       <c r="O41" s="9">
         <v>11</v>
       </c>
-    </row>
-    <row r="42" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P41" s="9">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A42" s="4">
         <v>37</v>
       </c>
@@ -2813,8 +2943,11 @@
       <c r="O42" s="8">
         <v>5</v>
       </c>
-    </row>
-    <row r="43" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P42" s="8">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A43" s="6">
         <v>38</v>
       </c>
@@ -2860,8 +2993,11 @@
       <c r="O43" s="9">
         <v>5</v>
       </c>
-    </row>
-    <row r="44" spans="1:15" ht="21" x14ac:dyDescent="0.3">
+      <c r="P43" s="9">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" ht="21" x14ac:dyDescent="0.3">
       <c r="A44" s="4">
         <v>39</v>
       </c>
@@ -2906,6 +3042,9 @@
       </c>
       <c r="O44" s="8">
         <v>6</v>
+      </c>
+      <c r="P44" s="8">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -2914,16 +3053,21 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <conditionalFormatting sqref="F6:J44">
-    <cfRule type="cellIs" dxfId="2" priority="5" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="6" stopIfTrue="1" operator="lessThan">
       <formula>10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6:K44">
-    <cfRule type="cellIs" dxfId="1" priority="6" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="7" stopIfTrue="1" operator="lessThan">
       <formula>2.5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L6:O44">
+    <cfRule type="cellIs" dxfId="1" priority="2" stopIfTrue="1" operator="lessThan">
+      <formula>10</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P6:P44">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="lessThan">
       <formula>10</formula>
     </cfRule>

</xml_diff>

<commit_message>
Add History (20pts) subject score to real_db.js and update index, leader, and parent pages
</commit_message>
<xml_diff>
--- a/Student_Midterm_Scores_M1_4.xlsx
+++ b/Student_Midterm_Scores_M1_4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\porsky\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06ABBCF1-3D5F-45D7-983D-6A1AF816EED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57365118-BD4B-4160-BDB4-51C1AA332318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="139">
   <si>
     <t>รายชื่อนักเรียนชั้นมัธยมศึกษาปีที่ 1.4 หลักสูตร SMT คะแนนสอบกลางภาค</t>
   </si>
@@ -454,6 +454,9 @@
   <si>
     <t>วิชาวิทยาศาสตร์
 ปฎิบัติการ</t>
+  </si>
+  <si>
+    <t>ประวัติศาสาตร์</t>
   </si>
 </sst>
 </file>
@@ -960,7 +963,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P44"/>
+  <dimension ref="A1:Q44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -975,9 +978,10 @@
     <col min="14" max="14" width="25.77734375" customWidth="1"/>
     <col min="15" max="15" width="21.6640625" customWidth="1"/>
     <col min="16" max="16" width="22.33203125" customWidth="1"/>
+    <col min="17" max="17" width="17.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="25.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" ht="25.8" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -992,7 +996,7 @@
       <c r="J1" s="11"/>
       <c r="K1" s="11"/>
     </row>
-    <row r="2" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -1007,7 +1011,7 @@
       <c r="J2" s="11"/>
       <c r="K2" s="11"/>
     </row>
-    <row r="4" spans="1:16" ht="21" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:17" ht="21" x14ac:dyDescent="0.4">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -1048,8 +1052,11 @@
       <c r="P4" s="2">
         <v>30</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="Q4" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1098,8 +1105,11 @@
       <c r="P5" s="3" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q5" s="3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>1</v>
       </c>
@@ -1148,8 +1158,11 @@
       <c r="P6" s="8">
         <v>21</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q6" s="8">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A7" s="6">
         <v>2</v>
       </c>
@@ -1198,8 +1211,11 @@
       <c r="P7" s="9">
         <v>23</v>
       </c>
-    </row>
-    <row r="8" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q7" s="9">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>3</v>
       </c>
@@ -1248,8 +1264,11 @@
       <c r="P8" s="8">
         <v>21</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q8" s="8">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A9" s="6">
         <v>4</v>
       </c>
@@ -1298,8 +1317,11 @@
       <c r="P9" s="9">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q9" s="9">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>5</v>
       </c>
@@ -1348,8 +1370,11 @@
       <c r="P10" s="8">
         <v>11</v>
       </c>
-    </row>
-    <row r="11" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q10" s="8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A11" s="6">
         <v>6</v>
       </c>
@@ -1396,8 +1421,11 @@
         <v>13</v>
       </c>
       <c r="P11" s="9"/>
-    </row>
-    <row r="12" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q11" s="9">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>7</v>
       </c>
@@ -1446,8 +1474,11 @@
       <c r="P12" s="8">
         <v>19</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q12" s="8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A13" s="6">
         <v>8</v>
       </c>
@@ -1496,8 +1527,11 @@
       <c r="P13" s="9">
         <v>14</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q13" s="9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>9</v>
       </c>
@@ -1546,8 +1580,11 @@
       <c r="P14" s="8">
         <v>20</v>
       </c>
-    </row>
-    <row r="15" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q14" s="8">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
         <v>10</v>
       </c>
@@ -1596,8 +1633,11 @@
       <c r="P15" s="9">
         <v>20</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q15" s="9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>11</v>
       </c>
@@ -1646,8 +1686,11 @@
       <c r="P16" s="8">
         <v>20</v>
       </c>
-    </row>
-    <row r="17" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q16" s="8">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
         <v>12</v>
       </c>
@@ -1696,8 +1739,11 @@
       <c r="P17" s="9">
         <v>18</v>
       </c>
-    </row>
-    <row r="18" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q17" s="9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>13</v>
       </c>
@@ -1746,8 +1792,11 @@
       <c r="P18" s="8">
         <v>19</v>
       </c>
-    </row>
-    <row r="19" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q18" s="8">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>14</v>
       </c>
@@ -1796,8 +1845,11 @@
       <c r="P19" s="9">
         <v>22</v>
       </c>
-    </row>
-    <row r="20" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q19" s="9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>15</v>
       </c>
@@ -1846,8 +1898,11 @@
       <c r="P20" s="8">
         <v>15</v>
       </c>
-    </row>
-    <row r="21" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q20" s="8">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A21" s="6">
         <v>16</v>
       </c>
@@ -1896,8 +1951,11 @@
       <c r="P21" s="9">
         <v>21</v>
       </c>
-    </row>
-    <row r="22" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q21" s="9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>17</v>
       </c>
@@ -1946,8 +2004,11 @@
       <c r="P22" s="8">
         <v>18</v>
       </c>
-    </row>
-    <row r="23" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q22" s="8">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A23" s="6">
         <v>18</v>
       </c>
@@ -1996,8 +2057,11 @@
       <c r="P23" s="9">
         <v>20</v>
       </c>
-    </row>
-    <row r="24" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q23" s="9">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
         <v>19</v>
       </c>
@@ -2046,8 +2110,11 @@
       <c r="P24" s="8">
         <v>19</v>
       </c>
-    </row>
-    <row r="25" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q24" s="8">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
         <v>20</v>
       </c>
@@ -2096,8 +2163,11 @@
       <c r="P25" s="9">
         <v>21</v>
       </c>
-    </row>
-    <row r="26" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q25" s="9">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
         <v>21</v>
       </c>
@@ -2146,8 +2216,11 @@
       <c r="P26" s="8">
         <v>19</v>
       </c>
-    </row>
-    <row r="27" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q26" s="8">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A27" s="6">
         <v>22</v>
       </c>
@@ -2196,8 +2269,11 @@
       <c r="P27" s="9">
         <v>19</v>
       </c>
-    </row>
-    <row r="28" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q27" s="9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A28" s="4">
         <v>23</v>
       </c>
@@ -2246,8 +2322,11 @@
       <c r="P28" s="8">
         <v>20</v>
       </c>
-    </row>
-    <row r="29" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q28" s="8">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A29" s="6">
         <v>24</v>
       </c>
@@ -2296,8 +2375,11 @@
       <c r="P29" s="9">
         <v>16</v>
       </c>
-    </row>
-    <row r="30" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q29" s="9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
         <v>25</v>
       </c>
@@ -2346,8 +2428,11 @@
       <c r="P30" s="8">
         <v>21</v>
       </c>
-    </row>
-    <row r="31" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q30" s="8">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A31" s="6">
         <v>26</v>
       </c>
@@ -2396,8 +2481,11 @@
       <c r="P31" s="9">
         <v>20</v>
       </c>
-    </row>
-    <row r="32" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q31" s="9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
         <v>27</v>
       </c>
@@ -2446,8 +2534,11 @@
       <c r="P32" s="8">
         <v>18</v>
       </c>
-    </row>
-    <row r="33" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q32" s="8">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A33" s="6">
         <v>28</v>
       </c>
@@ -2496,8 +2587,11 @@
       <c r="P33" s="9">
         <v>22</v>
       </c>
-    </row>
-    <row r="34" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q33" s="9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
         <v>29</v>
       </c>
@@ -2546,8 +2640,11 @@
       <c r="P34" s="8">
         <v>21</v>
       </c>
-    </row>
-    <row r="35" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q34" s="8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A35" s="6">
         <v>30</v>
       </c>
@@ -2596,8 +2693,11 @@
       <c r="P35" s="9">
         <v>20</v>
       </c>
-    </row>
-    <row r="36" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q35" s="9">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
         <v>31</v>
       </c>
@@ -2646,8 +2746,11 @@
       <c r="P36" s="8">
         <v>22</v>
       </c>
-    </row>
-    <row r="37" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q36" s="8">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A37" s="6">
         <v>32</v>
       </c>
@@ -2696,8 +2799,11 @@
       <c r="P37" s="9">
         <v>17</v>
       </c>
-    </row>
-    <row r="38" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q37" s="9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A38" s="4">
         <v>33</v>
       </c>
@@ -2746,8 +2852,11 @@
       <c r="P38" s="8">
         <v>23</v>
       </c>
-    </row>
-    <row r="39" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q38" s="8">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A39" s="6">
         <v>34</v>
       </c>
@@ -2796,8 +2905,11 @@
       <c r="P39" s="9">
         <v>20</v>
       </c>
-    </row>
-    <row r="40" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q39" s="9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
         <v>35</v>
       </c>
@@ -2846,8 +2958,11 @@
       <c r="P40" s="8">
         <v>21</v>
       </c>
-    </row>
-    <row r="41" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q40" s="8">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A41" s="6">
         <v>36</v>
       </c>
@@ -2896,8 +3011,11 @@
       <c r="P41" s="9">
         <v>24</v>
       </c>
-    </row>
-    <row r="42" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q41" s="9">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A42" s="4">
         <v>37</v>
       </c>
@@ -2946,8 +3064,11 @@
       <c r="P42" s="8">
         <v>22</v>
       </c>
-    </row>
-    <row r="43" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q42" s="8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A43" s="6">
         <v>38</v>
       </c>
@@ -2996,8 +3117,11 @@
       <c r="P43" s="9">
         <v>16</v>
       </c>
-    </row>
-    <row r="44" spans="1:16" ht="21" x14ac:dyDescent="0.3">
+      <c r="Q43" s="9">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" ht="21" x14ac:dyDescent="0.3">
       <c r="A44" s="4">
         <v>39</v>
       </c>
@@ -3045,6 +3169,9 @@
       </c>
       <c r="P44" s="8">
         <v>19</v>
+      </c>
+      <c r="Q44" s="8">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -3053,21 +3180,21 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <conditionalFormatting sqref="F6:J44">
-    <cfRule type="cellIs" dxfId="3" priority="6" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="7" stopIfTrue="1" operator="lessThan">
       <formula>10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6:K44">
-    <cfRule type="cellIs" dxfId="2" priority="7" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="8" stopIfTrue="1" operator="lessThan">
       <formula>2.5</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L6:O44">
+  <conditionalFormatting sqref="L6:P44">
     <cfRule type="cellIs" dxfId="1" priority="2" stopIfTrue="1" operator="lessThan">
       <formula>10</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P6:P44">
+  <conditionalFormatting sqref="Q6:Q44">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="lessThan">
       <formula>10</formula>
     </cfRule>

</xml_diff>

<commit_message>
Add Earth Science (40pts) score to real_db.js and update dashboard, leader, and parent portal pages
</commit_message>
<xml_diff>
--- a/Student_Midterm_Scores_M1_4.xlsx
+++ b/Student_Midterm_Scores_M1_4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\porsky\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57365118-BD4B-4160-BDB4-51C1AA332318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{706824AB-90F0-4970-853A-D4447A5D5B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="140">
   <si>
     <t>รายชื่อนักเรียนชั้นมัธยมศึกษาปีที่ 1.4 หลักสูตร SMT คะแนนสอบกลางภาค</t>
   </si>
@@ -457,6 +457,9 @@
   </si>
   <si>
     <t>ประวัติศาสาตร์</t>
+  </si>
+  <si>
+    <t>วิทยาศาสตร์โลกทั้งระบบ</t>
   </si>
 </sst>
 </file>
@@ -963,7 +966,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q44"/>
+  <dimension ref="A1:R44"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -979,9 +982,10 @@
     <col min="15" max="15" width="21.6640625" customWidth="1"/>
     <col min="16" max="16" width="22.33203125" customWidth="1"/>
     <col min="17" max="17" width="17.77734375" customWidth="1"/>
+    <col min="18" max="18" width="21.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="25.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="25.8" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -996,7 +1000,7 @@
       <c r="J1" s="11"/>
       <c r="K1" s="11"/>
     </row>
-    <row r="2" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -1011,7 +1015,7 @@
       <c r="J2" s="11"/>
       <c r="K2" s="11"/>
     </row>
-    <row r="4" spans="1:17" ht="21" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:18" ht="21" x14ac:dyDescent="0.4">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -1055,8 +1059,11 @@
       <c r="Q4" s="2">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="R4" s="2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -1108,8 +1115,11 @@
       <c r="Q5" s="3" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R5" s="3" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>1</v>
       </c>
@@ -1161,8 +1171,11 @@
       <c r="Q6" s="8">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R6" s="8">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A7" s="6">
         <v>2</v>
       </c>
@@ -1214,8 +1227,11 @@
       <c r="Q7" s="9">
         <v>16</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R7" s="9">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>3</v>
       </c>
@@ -1267,8 +1283,11 @@
       <c r="Q8" s="8">
         <v>12</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R8" s="8">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A9" s="6">
         <v>4</v>
       </c>
@@ -1320,8 +1339,11 @@
       <c r="Q9" s="9">
         <v>16</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R9" s="9">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>5</v>
       </c>
@@ -1373,8 +1395,11 @@
       <c r="Q10" s="8">
         <v>7</v>
       </c>
-    </row>
-    <row r="11" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R10" s="8">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A11" s="6">
         <v>6</v>
       </c>
@@ -1424,8 +1449,11 @@
       <c r="Q11" s="9">
         <v>16</v>
       </c>
-    </row>
-    <row r="12" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R11" s="9">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>7</v>
       </c>
@@ -1477,8 +1505,11 @@
       <c r="Q12" s="8">
         <v>15</v>
       </c>
-    </row>
-    <row r="13" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R12" s="8">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A13" s="6">
         <v>8</v>
       </c>
@@ -1530,8 +1561,11 @@
       <c r="Q13" s="9">
         <v>10</v>
       </c>
-    </row>
-    <row r="14" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R13" s="9">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>9</v>
       </c>
@@ -1583,8 +1617,11 @@
       <c r="Q14" s="8">
         <v>14</v>
       </c>
-    </row>
-    <row r="15" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R14" s="8">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A15" s="6">
         <v>10</v>
       </c>
@@ -1636,8 +1673,11 @@
       <c r="Q15" s="9">
         <v>15</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R15" s="9">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>11</v>
       </c>
@@ -1689,8 +1729,11 @@
       <c r="Q16" s="8">
         <v>7</v>
       </c>
-    </row>
-    <row r="17" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R16" s="8">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
         <v>12</v>
       </c>
@@ -1742,8 +1785,11 @@
       <c r="Q17" s="9">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R17" s="9">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>13</v>
       </c>
@@ -1795,8 +1841,11 @@
       <c r="Q18" s="8">
         <v>16</v>
       </c>
-    </row>
-    <row r="19" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R18" s="8">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
         <v>14</v>
       </c>
@@ -1848,8 +1897,11 @@
       <c r="Q19" s="9">
         <v>15</v>
       </c>
-    </row>
-    <row r="20" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R19" s="9">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A20" s="4">
         <v>15</v>
       </c>
@@ -1901,8 +1953,11 @@
       <c r="Q20" s="8">
         <v>16</v>
       </c>
-    </row>
-    <row r="21" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R20" s="8">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A21" s="6">
         <v>16</v>
       </c>
@@ -1954,8 +2009,11 @@
       <c r="Q21" s="9">
         <v>15</v>
       </c>
-    </row>
-    <row r="22" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R21" s="9">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A22" s="4">
         <v>17</v>
       </c>
@@ -2007,8 +2065,11 @@
       <c r="Q22" s="8">
         <v>9</v>
       </c>
-    </row>
-    <row r="23" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R22" s="8">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A23" s="6">
         <v>18</v>
       </c>
@@ -2060,8 +2121,11 @@
       <c r="Q23" s="9">
         <v>16</v>
       </c>
-    </row>
-    <row r="24" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R23" s="9">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A24" s="4">
         <v>19</v>
       </c>
@@ -2113,8 +2177,11 @@
       <c r="Q24" s="8">
         <v>16</v>
       </c>
-    </row>
-    <row r="25" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R24" s="8">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
         <v>20</v>
       </c>
@@ -2166,8 +2233,11 @@
       <c r="Q25" s="9">
         <v>11</v>
       </c>
-    </row>
-    <row r="26" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R25" s="9">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A26" s="4">
         <v>21</v>
       </c>
@@ -2219,8 +2289,11 @@
       <c r="Q26" s="8">
         <v>11</v>
       </c>
-    </row>
-    <row r="27" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R26" s="8">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A27" s="6">
         <v>22</v>
       </c>
@@ -2272,8 +2345,11 @@
       <c r="Q27" s="9">
         <v>15</v>
       </c>
-    </row>
-    <row r="28" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R27" s="9">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A28" s="4">
         <v>23</v>
       </c>
@@ -2325,8 +2401,11 @@
       <c r="Q28" s="8">
         <v>16</v>
       </c>
-    </row>
-    <row r="29" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R28" s="8">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A29" s="6">
         <v>24</v>
       </c>
@@ -2378,8 +2457,11 @@
       <c r="Q29" s="9">
         <v>8</v>
       </c>
-    </row>
-    <row r="30" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R29" s="9">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
         <v>25</v>
       </c>
@@ -2431,8 +2513,11 @@
       <c r="Q30" s="8">
         <v>16</v>
       </c>
-    </row>
-    <row r="31" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R30" s="8">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A31" s="6">
         <v>26</v>
       </c>
@@ -2484,8 +2569,11 @@
       <c r="Q31" s="9">
         <v>15</v>
       </c>
-    </row>
-    <row r="32" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R31" s="9">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
         <v>27</v>
       </c>
@@ -2537,8 +2625,11 @@
       <c r="Q32" s="8">
         <v>12</v>
       </c>
-    </row>
-    <row r="33" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R32" s="8">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A33" s="6">
         <v>28</v>
       </c>
@@ -2590,8 +2681,11 @@
       <c r="Q33" s="9">
         <v>15</v>
       </c>
-    </row>
-    <row r="34" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R33" s="9">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
         <v>29</v>
       </c>
@@ -2643,8 +2737,11 @@
       <c r="Q34" s="8">
         <v>15</v>
       </c>
-    </row>
-    <row r="35" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R34" s="8">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A35" s="6">
         <v>30</v>
       </c>
@@ -2696,8 +2793,11 @@
       <c r="Q35" s="9">
         <v>11</v>
       </c>
-    </row>
-    <row r="36" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R35" s="9">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
         <v>31</v>
       </c>
@@ -2749,8 +2849,11 @@
       <c r="Q36" s="8">
         <v>12</v>
       </c>
-    </row>
-    <row r="37" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R36" s="8">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A37" s="6">
         <v>32</v>
       </c>
@@ -2802,8 +2905,11 @@
       <c r="Q37" s="9">
         <v>10</v>
       </c>
-    </row>
-    <row r="38" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R37" s="9">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A38" s="4">
         <v>33</v>
       </c>
@@ -2855,8 +2961,11 @@
       <c r="Q38" s="8">
         <v>17</v>
       </c>
-    </row>
-    <row r="39" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R38" s="8">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A39" s="6">
         <v>34</v>
       </c>
@@ -2908,8 +3017,11 @@
       <c r="Q39" s="9">
         <v>10</v>
       </c>
-    </row>
-    <row r="40" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R39" s="9">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
         <v>35</v>
       </c>
@@ -2961,8 +3073,11 @@
       <c r="Q40" s="8">
         <v>16</v>
       </c>
-    </row>
-    <row r="41" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R40" s="8">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A41" s="6">
         <v>36</v>
       </c>
@@ -3014,8 +3129,11 @@
       <c r="Q41" s="9">
         <v>15</v>
       </c>
-    </row>
-    <row r="42" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R41" s="9">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A42" s="4">
         <v>37</v>
       </c>
@@ -3067,8 +3185,11 @@
       <c r="Q42" s="8">
         <v>15</v>
       </c>
-    </row>
-    <row r="43" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R42" s="8">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A43" s="6">
         <v>38</v>
       </c>
@@ -3120,8 +3241,11 @@
       <c r="Q43" s="9">
         <v>13</v>
       </c>
-    </row>
-    <row r="44" spans="1:17" ht="21" x14ac:dyDescent="0.3">
+      <c r="R43" s="9">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" ht="21" x14ac:dyDescent="0.3">
       <c r="A44" s="4">
         <v>39</v>
       </c>
@@ -3172,6 +3296,9 @@
       </c>
       <c r="Q44" s="8">
         <v>11</v>
+      </c>
+      <c r="R44" s="8">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -3180,21 +3307,21 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <conditionalFormatting sqref="F6:J44">
-    <cfRule type="cellIs" dxfId="3" priority="7" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="3" priority="8" stopIfTrue="1" operator="lessThan">
       <formula>10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6:K44">
-    <cfRule type="cellIs" dxfId="2" priority="8" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="9" stopIfTrue="1" operator="lessThan">
       <formula>2.5</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L6:P44">
+  <conditionalFormatting sqref="L6:Q44">
     <cfRule type="cellIs" dxfId="1" priority="2" stopIfTrue="1" operator="lessThan">
       <formula>10</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q6:Q44">
+  <conditionalFormatting sqref="R6:R44">
     <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="lessThan">
       <formula>10</formula>
     </cfRule>

</xml_diff>